<commit_message>
Marketing: record Marketing Services queue ID 13519272 (confirmed)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FjvmSq7K8pjfTvM6rQ1ZUn
</commit_message>
<xml_diff>
--- a/audits/marketing-workflow-audit/WLS_Marketing_Workflow_Audit.xlsx
+++ b/audits/marketing-workflow-audit/WLS_Marketing_Workflow_Audit.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed Action Map'!$A$1:$S$90</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Task &amp; Subtask Logic'!$A$1:$Q$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Workflow Inventory'!$A$1:$K$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Audit Findings'!$A$1:$I$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Audit Findings'!$A$1:$I$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -12824,7 +12824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -13455,14 +13455,14 @@
           <t>F-13</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Needs Verification</t>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>No Issue Found</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>All three workflows</t>
+          <t>All in scope</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -13472,22 +13472,22 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>All 24 Create task actions use queue ID 13519272. HubSpot doesn't return queue names through the API, so it isn't confirmed that this ID is the "Marketing Services" queue. (It differs from the Ops Tasks queue, 13519269.)</t>
+          <t>Every Create task action in every in-scope workflow uses the team queue (13519272).</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>VERIFIED (config): queue_id 13519272 on every Create task action.</t>
+          <t>Config queue_id on every Create task action.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>The "every task uses the Marketing Services queue" check (F-14) relies on this ID being that queue.</t>
+          <t>Confirms the rule.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Open the Marketing Services queue in HubSpot and confirm its ID is 13519272, then record it in teams.json.</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -13514,17 +13514,17 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Create task actions</t>
+          <t>Tasks</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Every Create task action in every in-scope workflow uses the team queue (13519272).</t>
+          <t>No task has been created on or after 2026-10-06 by any in-scope workflow that is now switched off.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Config queue_id on every Create task action.</t>
+          <t>Task records by workflow name, start date onward.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -13566,12 +13566,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>No task has been created on or after 2026-10-06 by any in-scope workflow that is now switched off.</t>
+          <t>No company received the same task twice on the same day since 2026-10-06.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Task records by workflow name, start date onward.</t>
+          <t>Task records: company + task title + creation date.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -13590,55 +13590,8 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>F-16</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>No Issue Found</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>All in scope</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Tasks</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>No company received the same task twice on the same day since 2026-10-06.</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Task records: company + task title + creation date.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Confirms the rule.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I17"/>
+  <autoFilter ref="A1:I16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>